<commit_message>
create folders under c:\Fatina
</commit_message>
<xml_diff>
--- a/BOQ.xlsx
+++ b/BOQ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ares\___projects___\Johnkh69\Python-React\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83BF6F74-554D-4B5C-A30A-85C1836A46B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{070FB071-535B-4443-9748-ADE941CF0AD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{B65C2978-E994-4025-97B3-A1A61B437853}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{B65C2978-E994-4025-97B3-A1A61B437853}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="144">
   <si>
     <t xml:space="preserve">Serial Number </t>
   </si>
@@ -454,6 +454,9 @@
   </si>
   <si>
     <t>System</t>
+  </si>
+  <si>
+    <t>01.02.02.2275</t>
   </si>
 </sst>
 </file>
@@ -4282,14 +4285,59 @@
       <c r="R61" s="21"/>
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A62" s="1"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="3"/>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1"/>
-      <c r="H62" s="1"/>
-      <c r="I62" s="1"/>
+      <c r="A62" s="13">
+        <v>61</v>
+      </c>
+      <c r="B62" s="13">
+        <v>1</v>
+      </c>
+      <c r="C62" s="13">
+        <v>3</v>
+      </c>
+      <c r="D62" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E62" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="F62" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G62" s="16">
+        <v>5</v>
+      </c>
+      <c r="H62" s="17">
+        <v>3969.0000000000005</v>
+      </c>
+      <c r="I62" s="18">
+        <f t="shared" ref="I62" si="2">H62*G62</f>
+        <v>19845.000000000004</v>
+      </c>
+      <c r="J62" s="19">
+        <v>0</v>
+      </c>
+      <c r="K62" s="19">
+        <v>0</v>
+      </c>
+      <c r="L62" s="20">
+        <v>0</v>
+      </c>
+      <c r="M62" s="20">
+        <v>0</v>
+      </c>
+      <c r="N62" s="18">
+        <v>0</v>
+      </c>
+      <c r="O62" s="18">
+        <v>0</v>
+      </c>
+      <c r="P62" s="18">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="18">
+        <v>0</v>
+      </c>
+      <c r="R62" s="21"/>
     </row>
     <row r="63" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
@@ -4306,25 +4354,25 @@
       <c r="J63" s="4"/>
       <c r="K63" s="4"/>
       <c r="N63" s="18">
-        <f t="shared" ref="N63:Q63" si="2">SUBTOTAL(9,N2:N61)</f>
+        <f t="shared" ref="N63:Q63" si="3">SUBTOTAL(9,N2:N61)</f>
         <v>5736042.8316000002</v>
       </c>
       <c r="O63" s="18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3470439.6540000001</v>
       </c>
       <c r="P63" s="18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q63" s="18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange sqref="G8:G61 G2:G6" name="Price_3_1_1_1"/>
+    <protectedRange sqref="G2:G6 G8:G62" name="Price_3_1_1_1"/>
     <protectedRange sqref="G7" name="Price_3_2_1_1"/>
   </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>